<commit_message>
working on field selection prioroities
</commit_message>
<xml_diff>
--- a/fieldSelectionPriorityList.xlsx
+++ b/fieldSelectionPriorityList.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Career\00. Univesity\PHD\5. Field selection\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Career\00. Univesity\PHD\2. Exam Log\blackoutPhdPreparation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47F48ACA-2D7B-4520-9B76-3593B85D7BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A1D4F5F-27FD-42EA-A721-C265D4AEE8ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C41F7097-CAB5-4071-B473-853C504AEB75}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="70">
   <si>
     <t>Priority</t>
   </si>
@@ -522,37 +522,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -572,6 +551,27 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1251,223 +1251,223 @@
   <sheetData>
     <row r="1" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6" t="s">
+      <c r="D2" s="15"/>
+      <c r="E2" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="F2" s="7"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="3" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="11" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="4" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C4" s="10">
+      <c r="C4" s="20">
         <v>1</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="18">
         <f>C11+1</f>
         <v>9</v>
       </c>
-      <c r="F4" s="19" t="s">
-        <v>61</v>
+      <c r="F4" s="12" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="5" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C5" s="10">
+      <c r="C5" s="20">
         <v>2</v>
       </c>
-      <c r="D5" s="16" t="s">
+      <c r="D5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="18">
         <f>E4+1</f>
         <v>10</v>
       </c>
-      <c r="F5" s="19" t="s">
-        <v>5</v>
+      <c r="F5" s="12" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C6" s="10">
+      <c r="C6" s="20">
         <v>3</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="18">
         <f t="shared" ref="E6:E18" si="0">E5+1</f>
         <v>11</v>
       </c>
-      <c r="F6" s="19" t="s">
+      <c r="F6" s="12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C7" s="20">
+        <v>4</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="18">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C8" s="20">
+        <v>5</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="18">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C9" s="20">
+        <v>6</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="18">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C10" s="20">
+        <v>7</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="18">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C11" s="20">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C7" s="10">
-        <v>4</v>
-      </c>
-      <c r="D7" s="16" t="s">
+      <c r="D11" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E11" s="18">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C12" s="6"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="18">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C13" s="6"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="18">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="14" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C14" s="6"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="18">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C15" s="6"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="18">
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="E7" s="11">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C8" s="10">
-        <v>5</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="11">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="F8" s="19" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C9" s="10">
-        <v>6</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="11">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="F9" s="19" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C10" s="10">
-        <v>7</v>
-      </c>
-      <c r="D10" s="16" t="s">
+      <c r="F15" s="12" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C16" s="6"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="18">
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="E10" s="11">
-        <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="F10" s="19" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C11" s="10">
-        <v>8</v>
-      </c>
-      <c r="D11" s="16" t="s">
+      <c r="F16" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C17" s="6"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="18">
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="E11" s="11">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="F11" s="19" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C12" s="12"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="11">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-      <c r="F12" s="19" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="13" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C13" s="12"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="11">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-      <c r="F13" s="19" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C14" s="12"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="11">
-        <f t="shared" si="0"/>
-        <v>19</v>
-      </c>
-      <c r="F14" s="19" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="15" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C15" s="12"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="11">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="F15" s="19" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="16" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C16" s="12"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="11">
-        <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
-      <c r="F16" s="19" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="17" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C17" s="12"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="11">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-      <c r="F17" s="19" t="s">
+      <c r="F17" s="12" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="18" spans="3:6" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C18" s="13"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="14">
+      <c r="C18" s="7"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="19">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="F18" s="20" t="s">
+      <c r="F18" s="13" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>